<commit_message>
updated the paper and added latex code
</commit_message>
<xml_diff>
--- a/Results/panel_model_res.xlsx
+++ b/Results/panel_model_res.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11113"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victoryerz/Desktop/GaR-project/results/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67C6E64-7724-2E4E-9822-01FD992D58AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t>GDP growth, h=4, q=0.1, e=f</t>
   </si>
@@ -317,16 +311,13 @@
   </si>
   <si>
     <t>(0.0913)</t>
-  </si>
-  <si>
-    <t>Variables</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,36 +326,23 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="9"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -374,87 +352,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -462,35 +369,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -498,14 +380,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -552,7 +426,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -584,27 +458,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -636,24 +492,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -829,424 +667,417 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="28.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="18.83203125" style="1" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B1" s="7" t="s">
+    <row r="1" spans="1:3">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:3">
+      <c r="A3" s="1"/>
+      <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:3">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="1:3">
+      <c r="A5" s="1"/>
+      <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:3">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="2" t="s">
+    <row r="7" spans="1:3">
+      <c r="A7" s="1"/>
+      <c r="B7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:3">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
-      <c r="B9" s="2" t="s">
+    <row r="9" spans="1:3">
+      <c r="A9" s="1"/>
+      <c r="B9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:3">
+      <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="3"/>
-      <c r="B11" s="2" t="s">
+    <row r="11" spans="1:3">
+      <c r="A11" s="1"/>
+      <c r="B11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:3">
+      <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2" t="s">
+    <row r="13" spans="1:3">
+      <c r="A13" s="1"/>
+      <c r="B13" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:3">
+      <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
-      <c r="B15" s="2" t="s">
+    <row r="15" spans="1:3">
+      <c r="A15" s="1"/>
+      <c r="B15" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:3">
+      <c r="A16" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
-      <c r="B17" s="2" t="s">
+    <row r="17" spans="1:3">
+      <c r="A17" s="1"/>
+      <c r="B17" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:3">
+      <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="3"/>
-      <c r="B19" s="2" t="s">
+    <row r="19" spans="1:3">
+      <c r="A19" s="1"/>
+      <c r="B19" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="B21" s="2" t="s">
+    <row r="21" spans="1:3">
+      <c r="A21" s="1"/>
+      <c r="B21" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:3">
+      <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
-      <c r="B23" s="2" t="s">
+    <row r="23" spans="1:3">
+      <c r="A23" s="1"/>
+      <c r="B23" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:3">
+      <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="3"/>
-      <c r="B25" s="2" t="s">
+    <row r="25" spans="1:3">
+      <c r="A25" s="1"/>
+      <c r="B25" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:3">
+      <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="3"/>
-      <c r="B27" s="2" t="s">
+    <row r="27" spans="1:3">
+      <c r="A27" s="1"/>
+      <c r="B27" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:3">
+      <c r="A28" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" t="s">
         <v>49</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="3"/>
-      <c r="B29" s="2" t="s">
+    <row r="29" spans="1:3">
+      <c r="A29" s="1"/>
+      <c r="B29" t="s">
         <v>50</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:3">
+      <c r="A30" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" t="s">
         <v>51</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="3"/>
-      <c r="B31" s="2" t="s">
+    <row r="31" spans="1:3">
+      <c r="A31" s="1"/>
+      <c r="B31" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:3">
+      <c r="A32" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" t="s">
         <v>53</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="3"/>
-      <c r="B33" s="2" t="s">
+    <row r="33" spans="1:3">
+      <c r="A33" s="1"/>
+      <c r="B33" t="s">
         <v>54</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:3">
+      <c r="A34" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="3"/>
-      <c r="B35" s="2" t="s">
+    <row r="35" spans="1:3">
+      <c r="A35" s="1"/>
+      <c r="B35" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
+    <row r="36" spans="1:3">
+      <c r="A36" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" t="s">
         <v>57</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
-      <c r="B37" s="2" t="s">
+    <row r="37" spans="1:3">
+      <c r="A37" s="1"/>
+      <c r="B37" t="s">
         <v>58</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:3">
+      <c r="A38" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" t="s">
         <v>59</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="3"/>
-      <c r="B39" s="2" t="s">
+    <row r="39" spans="1:3">
+      <c r="A39" s="1"/>
+      <c r="B39" t="s">
         <v>60</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
+    <row r="40" spans="1:3">
+      <c r="A40" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40">
         <v>4469</v>
       </c>
-      <c r="C40" s="4">
+      <c r="C40">
         <v>4469</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
+    <row r="41" spans="1:3">
+      <c r="A41" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B41" s="9">
+      <c r="B41">
         <v>0.1831110064914544</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41">
         <v>0.2007309044629306</v>
       </c>
     </row>

</xml_diff>